<commit_message>
mostrar cantidad de productos por categoria y proveedor
- Añade migración `008_entity_product_counts.sql` con las vistas `categories_with_counts` y `suppliers_with_counts`.
- Actualiza tipos de la base de datos y define alias `CategoryWithCount` y `SupplierWithCount`.
- Modifica las Server Actions `getCategories` y `getSuppliers` para consumir las nuevas vistas.
- Agrega columna de "Productos" ordenable en las tablas cliente de Categorías y Proveedores.
</commit_message>
<xml_diff>
--- a/documentacion/Matriz de casos de prueba.xlsx
+++ b/documentacion/Matriz de casos de prueba.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DCB74169-975F-4A03-BC34-AEDDF9B4720A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC40F387-DCCE-411D-B3AA-536B5CB1C21E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="3" r:id="rId1"/>
@@ -15,6 +15,9 @@
     <sheet name="Categorias" sheetId="5" r:id="rId5"/>
     <sheet name="Proveedores" sheetId="6" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="J1K1">Dashboard!$J$1:$J$1</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -38,31 +41,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={8E1B78E2-7D98-4C60-96A8-B2B43EEF13EB}</author>
-  </authors>
-  <commentList>
-    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{8E1B78E2-7D98-4C60-96A8-B2B43EEF13EB}">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-[Tasks]
-There is a task anchored to this comment that cannot be viewed in your client.
-Comment:
-    @CIFUENTES LATRELLE MATIAS GABRIEL
-Reply:
-    hola
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="154">
   <si>
     <t>ID</t>
   </si>
@@ -333,9 +313,7 @@
     <t>Tooltip del gráfico de líneas Movimientos últimos 30 días</t>
   </si>
   <si>
-    <t>1- Acceder al módulo de Dashboard.
-2- Posicionar el cursor sobre algún punto de cualquiera de las líneas del gráfico Movimientos últimos 30 días.
-3- Visualizar el tooltip emergente.</t>
+    <t>1- Acceder al módulo de Dashboard. 2- Posicionar el cursor sobre algún punto de cualquiera de las líneas del gráfico Movimientos últimos 30 días. 3- Visualizar el tooltip emergente.</t>
   </si>
   <si>
     <t>Al hacer hover sobre el gráfico de líneas debe aparecer un tooltip mostrando la fecha y los valores de Ajustes, Entradas y Salidas correspondientes a esa fecha.</t>
@@ -364,6 +342,24 @@
   </si>
   <si>
     <t>El sistema redirige al modulo de Categorias.</t>
+  </si>
+  <si>
+    <t>DB-007</t>
+  </si>
+  <si>
+    <t>Verificar mensaje de bienvenida con usuario Admin</t>
+  </si>
+  <si>
+    <t>Ingresar a https://challenge-tecnico-aranguri-apps.vercel.app/ con credenciales: Mail: Admin@email.com Password: Admin123</t>
+  </si>
+  <si>
+    <t>1- Acceder al modulo de Dashboard. 2- Visualizar el mensaje de bienvenida en la parte superior de la pantalla.</t>
+  </si>
+  <si>
+    <t>El sistema muestra el mensaje de bienvenida correspondiente al usuario Admin, con el saludo segun la hora del dia y el subtitulo Resumen general del inventario.</t>
+  </si>
+  <si>
+    <t>El sistema muestra correctamente el mensaje Buenas tardes, Admin y el subtitulo Resumen general del inventario.</t>
   </si>
   <si>
     <t>PR-001</t>
@@ -462,6 +458,42 @@
     <t>La grilla muestra el mensaje "Sin productos Agregá tu primer producto al inventario"</t>
   </si>
   <si>
+    <t>PR-003</t>
+  </si>
+  <si>
+    <t>Agregar nuevo producto exitosamente</t>
+  </si>
+  <si>
+    <t>Ingresar a https://challenge-tecnico-aranguri-apps.vercel.app/ con credenciales: Mail: Admin@email.com Password: Admin123. Navegar al modulo de Productos.</t>
+  </si>
+  <si>
+    <t>1- Hacer click en el boton Nuevo producto. 2- Completar el campo Nombre con un valor valido (ej: Casco Protector). 3- Seleccionar una Unidad (ej: unidad). 4- Ingresar Precio unitario (ej: 5000). 5- Dejar Stock minimo en 5. 6- Hacer click en Guardar producto.</t>
+  </si>
+  <si>
+    <t>El producto se guarda exitosamente y aparece en la grilla de Productos.</t>
+  </si>
+  <si>
+    <t>El producto Casco Protector se guarda y aparece en la grilla.</t>
+  </si>
+  <si>
+    <t>PR-004</t>
+  </si>
+  <si>
+    <t>Verificar UI del formulario Nuevo producto</t>
+  </si>
+  <si>
+    <t>1- Hacer click en el boton Nuevo producto. 2- Verificar que el panel lateral se despliega correctamente. 3- Verificar que los campos Nombre, SKU, Unidad, Categoria, Proveedor, Precio unitario, Stock minimo y Descripcion son visibles. 4- Verificar que los campos obligatorios esten marcados con asterisco. 5- Verificar que el boton Guardar producto tiene el color brand (amarillo).</t>
+  </si>
+  <si>
+    <t>El panel lateral se despliega correctamente. Todos los campos son visibles y los obligatorios estan marcados con asterisco (*). El boton Guardar producto se muestra en color amarillo (color brand de la aplicacion).</t>
+  </si>
+  <si>
+    <t>El panel se despliega correctamente, todos los campos son visibles, los obligatorios tienen asterisco y el boton es amarillo.</t>
+  </si>
+  <si>
+    <t>UI</t>
+  </si>
+  <si>
     <t>MOV-001</t>
   </si>
   <si>
@@ -529,6 +561,24 @@
     <t>Se descarga correctamente un archivo Excel con todos los movimientos registrados en la grilla, con las columnas Fecha, Producto, SKU, Tipo, Cantidad, Motivo y Referencia.</t>
   </si>
   <si>
+    <t>MOV-003</t>
+  </si>
+  <si>
+    <t>Registrar nuevo movimiento de Entrada exitosamente</t>
+  </si>
+  <si>
+    <t>Ingresar a https://challenge-tecnico-aranguri-apps.vercel.app/ con credenciales: Mail: Admin@email.com Password: Admin123. Navegar al modulo de Movimientos.</t>
+  </si>
+  <si>
+    <t>1- Hacer click en Registrar movimiento. 2- Seleccionar un producto (ej: Multimetro Digital UNI-T). 3- Seleccionar Tipo: Entrada. 4- Ingresar Cantidad: 10. 5- Ingresar Motivo: Compra insumos. 6- Hacer click en Registrar movimiento.</t>
+  </si>
+  <si>
+    <t>El movimiento se registra exitosamente y aparece en la grilla con el tipo Entrada, el producto y la cantidad indicados.</t>
+  </si>
+  <si>
+    <t>El movimiento Entrada de Multimetro Digital UNI-T por 10 unidades se registra y aparece en la grilla.</t>
+  </si>
+  <si>
     <t>CAT-001</t>
   </si>
   <si>
@@ -648,6 +698,24 @@
     <t>Se visualiza correctamente la grilla ordenada de forma ascendente segun la columna Descripcion.</t>
   </si>
   <si>
+    <t>CAT-004</t>
+  </si>
+  <si>
+    <t>Agregar nueva categoria exitosamente</t>
+  </si>
+  <si>
+    <t>Ingresar a https://challenge-tecnico-aranguri-apps.vercel.app/ con credenciales: Mail: Admin@email.com Password: Admin123. Navegar al modulo de Categorias.</t>
+  </si>
+  <si>
+    <t>1- Hacer click en el boton Nueva categoria. 2- Completar el campo Nombre (ej: Seguridad). 3- Seleccionar un color (ej: verde). 4- Ingresar Descripcion (ej: Equipos de seguridad). 5- Hacer click en Guardar categoria.</t>
+  </si>
+  <si>
+    <t>La categoria se guarda exitosamente y aparece en la grilla de Categorias con el nombre, color y descripcion indicados.</t>
+  </si>
+  <si>
+    <t>La categoria Seguridad se guarda y aparece en la grilla con el color y descripcion correctos. Y queda asginable a productos</t>
+  </si>
+  <si>
     <t>PROV-001</t>
   </si>
   <si>
@@ -701,6 +769,24 @@
   </si>
   <si>
     <t>Se visualiza correctamente la grilla ordenada de forma ascendente por Contacto: Probado (–), HerraMax SRL (Ana González), Insumos Norte (Diego Peralta), TechDistrib SA (Marcelo Ruiz).</t>
+  </si>
+  <si>
+    <t>PROV-004</t>
+  </si>
+  <si>
+    <t>Agregar nuevo proveedor exitosamente</t>
+  </si>
+  <si>
+    <t>Ingresar a https://challenge-tecnico-aranguri-apps.vercel.app/ con credenciales: Mail: Admin@email.com Password: Admin123. Navegar al modulo de Proveedores.</t>
+  </si>
+  <si>
+    <t>1- Hacer click en el boton Nuevo proveedor. 2- Completar el campo Nombre (ej: Distribuidora Sur SA). 3- Ingresar Persona de contacto (ej: Laura Gomez). 4- Ingresar Email (ej: laura@distribuidorasur.com.ar). 5- Ingresar Telefono (ej: 011-4321-9876). 6- Hacer click en Guardar proveedor.</t>
+  </si>
+  <si>
+    <t>El proveedor se guarda exitosamente y aparece en la grilla de Proveedores con los datos ingresados.</t>
+  </si>
+  <si>
+    <t>El proveedor Distribuidora Sur SA se guarda y aparece en la grilla con el contacto, email y telefono correctos.</t>
   </si>
 </sst>
 </file>
@@ -971,7 +1057,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1025,9 +1111,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1074,9 +1157,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1176,6 +1256,19 @@
     <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1199,39 +1292,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
-<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks">
-  <Task id="{C5332195-6D33-4952-B962-6E3F7B5C6FDE}">
-    <Anchor>
-      <Comment id="{8E1B78E2-7D98-4C60-96A8-B2B43EEF13EB}"/>
-    </Anchor>
-    <History>
-      <Event time="2026-06-27T22:40:15.86" id="{1AC6A538-3F9F-48DC-9F37-3000807FB5E4}">
-        <Attribution userId="S::paltamiranda987@alumno.unlam.edu.ar::5de0030f-4e27-4118-b71e-f9dbe66d066b" userName="ALTAMIRANDA PATRICIO SEBASTIAN" userProvider="AD"/>
-        <Anchor>
-          <Comment id="{8E1B78E2-7D98-4C60-96A8-B2B43EEF13EB}"/>
-        </Anchor>
-        <Create/>
-      </Event>
-      <Event time="2026-06-27T22:40:15.86" id="{53ABBC5A-9267-4A62-A3FD-34C29BD9B02A}">
-        <Attribution userId="S::paltamiranda987@alumno.unlam.edu.ar::5de0030f-4e27-4118-b71e-f9dbe66d066b" userName="ALTAMIRANDA PATRICIO SEBASTIAN" userProvider="AD"/>
-        <Anchor>
-          <Comment id="{8E1B78E2-7D98-4C60-96A8-B2B43EEF13EB}"/>
-        </Anchor>
-        <Assign userId="S::mcifuenteslatrelle748@alumno.unlam.edu.ar::2378ef2b-5104-4a32-ba14-e94bc1779d78" userName="CIFUENTES LATRELLE MATIAS GABRIEL" userProvider="AD"/>
-      </Event>
-      <Event time="2026-06-27T22:40:15.86" id="{1E2348DF-0AC1-499A-A887-6F48E6D5F13B}">
-        <Attribution userId="S::paltamiranda987@alumno.unlam.edu.ar::5de0030f-4e27-4118-b71e-f9dbe66d066b" userName="ALTAMIRANDA PATRICIO SEBASTIAN" userProvider="AD"/>
-        <Anchor>
-          <Comment id="{8E1B78E2-7D98-4C60-96A8-B2B43EEF13EB}"/>
-        </Anchor>
-        <SetTitle title="@CIFUENTES LATRELLE MATIAS GABRIEL"/>
-      </Event>
-    </History>
-  </Task>
-</Tasks>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1658,6 +1718,53 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>3133725</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1209675</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7D6E3768-50E7-D321-DC1E-747AEDCE56CD}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{FFC909F6-5729-3779-EEA1-7E1F78CF553C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17849850" y="10220325"/>
+          <a:ext cx="2752725" cy="1209675"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1754,6 +1861,100 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2533650</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>1295400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6B69DA09-D845-3B2F-503F-FFBE70F6353D}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{B04ED236-7099-4BB3-BD9B-3E4D400942AA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17640300" y="2876550"/>
+          <a:ext cx="2381250" cy="1257300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>295275</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2667000</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1695450</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B8266857-4D10-783D-A078-062E718D15DF}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{6B69DA09-D845-3B2F-503F-FFBE70F6353D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17506950" y="4486275"/>
+          <a:ext cx="2647950" cy="1400175"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1850,6 +2051,100 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1457325</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>1857375</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F684F9A4-E733-4A61-3996-C9F1B870A060}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{002C3B70-14E1-2CFB-2954-C0FDBE6542BB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18621375" y="3171825"/>
+          <a:ext cx="1304925" cy="1809750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1485900</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>485775</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>3276600</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>1381125</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Imagen 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{18C73708-C7A6-BD07-C2B5-2BAFCC295579}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{F684F9A4-E733-4A61-3996-C9F1B870A060}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19954875" y="3609975"/>
+          <a:ext cx="1790700" cy="895350"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1858,15 +2153,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>161925</xdr:colOff>
+      <xdr:colOff>647700</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>95250</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>4095750</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>1724025</xdr:rowOff>
+      <xdr:rowOff>1733550</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1889,7 +2184,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16221075" y="285750"/>
+          <a:off x="18087975" y="295275"/>
           <a:ext cx="3448050" cy="1695450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1902,15 +2197,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
+      <xdr:colOff>647700</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>57150</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>4086225</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>1714500</xdr:rowOff>
+      <xdr:rowOff>1743075</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1936,7 +2231,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17573625" y="2066925"/>
+          <a:off x="18087975" y="2095500"/>
           <a:ext cx="3438525" cy="1685925"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1949,15 +2244,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>142875</xdr:colOff>
+      <xdr:colOff>600075</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>57150</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>4029075</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>1743075</xdr:rowOff>
+      <xdr:rowOff>1714500</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1983,8 +2278,102 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17583150" y="3914775"/>
+          <a:off x="18040350" y="3886200"/>
           <a:ext cx="3429000" cy="1685925"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>428625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2076450</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1333500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6F217CFB-682F-C14A-F40F-215822F29AC6}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{3513B811-B5DD-92AE-510E-15B6DD6273C8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17497425" y="6143625"/>
+          <a:ext cx="2019300" cy="904875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2924175</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>4124325</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1685925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Imagen 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B4A18541-5570-7426-B50C-0ACD31CB7EB5}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{6F217CFB-682F-C14A-F40F-215822F29AC6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="20364450" y="5753100"/>
+          <a:ext cx="1200150" cy="1647825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2136,14 +2525,101 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2076450</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>3295650</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1905000</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E513FC66-3F06-6199-5ECB-A621A59A3F07}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{9613D006-58D6-3569-D696-888FD178E5F3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18135600" y="5162550"/>
+          <a:ext cx="1219200" cy="1809750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>819150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2009775</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1323975</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Imagen 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{68E3BFDF-B6F8-F2AC-B1EE-C21B02EAA258}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{E513FC66-3F06-6199-5ECB-A621A59A3F07}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="16154400" y="5886450"/>
+          <a:ext cx="1914525" cy="504825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="CIFUENTES LATRELLE MATIAS GABRIEL" id="{B50D9BD7-368E-409A-B26F-55F05917D7F3}" userId="mcifuenteslatrelle748@alumno.unlam.edu.ar" providerId="PeoplePicker"/>
-  <person displayName="ALTAMIRANDA PATRICIO SEBASTIAN" id="{662202F7-865F-4991-A720-D4907830BBB6}" userId="S::paltamiranda987@alumno.unlam.edu.ar::5de0030f-4e27-4118-b71e-f9dbe66d066b" providerId="AD"/>
-</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2441,21 +2917,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="E3" dT="2026-06-27T22:40:17.01" personId="{662202F7-865F-4991-A720-D4907830BBB6}" id="{8E1B78E2-7D98-4C60-96A8-B2B43EEF13EB}">
-    <text>@CIFUENTES LATRELLE MATIAS GABRIEL</text>
-    <mentions>
-      <mention mentionpersonId="{B50D9BD7-368E-409A-B26F-55F05917D7F3}" mentionId="{A938E611-330E-4649-A325-4CA7D7F35C46}" startIndex="0" length="34"/>
-    </mentions>
-  </threadedComment>
-  <threadedComment ref="E3" dT="2026-06-27T22:40:24.26" personId="{662202F7-865F-4991-A720-D4907830BBB6}" id="{45DD19CE-C460-4EC9-8A26-470C18A283C9}" parentId="{8E1B78E2-7D98-4C60-96A8-B2B43EEF13EB}">
-    <text xml:space="preserve">hola
-</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1071EF2-3E39-441E-A0A9-CEDA178FF542}">
   <dimension ref="A1:L3"/>
@@ -2487,10 +2948,10 @@
       <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="20" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="6" t="s">
@@ -2513,73 +2974,73 @@
       </c>
     </row>
     <row r="2" spans="1:12" ht="147" customHeight="1">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="59" t="s">
+      <c r="C2" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="D2" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="31" t="s">
+      <c r="E2" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="70" t="s">
+      <c r="F2" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="30" t="s">
+      <c r="G2" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="30" t="s">
+      <c r="H2" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="34">
+      <c r="I2" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="33">
         <v>46201</v>
       </c>
-      <c r="L2" s="22"/>
+      <c r="L2" s="21"/>
     </row>
     <row r="3" spans="1:12" ht="117.75" customHeight="1">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="60" t="s">
+      <c r="C3" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="61" t="s">
+      <c r="D3" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="62" t="s">
+      <c r="F3" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="G3" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="29">
+      <c r="I3" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="28">
         <v>46202</v>
       </c>
       <c r="L3" s="4"/>
@@ -2591,7 +3052,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2610,132 +3071,132 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="17.25">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="41" t="s">
+      <c r="D1" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="42" t="s">
+      <c r="E1" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="42" t="s">
+      <c r="F1" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="41" t="s">
+      <c r="G1" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="40" t="s">
+      <c r="H1" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="40" t="s">
+      <c r="I1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="40" t="s">
+      <c r="J1" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="41" t="s">
+      <c r="K1" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="65" t="s">
+      <c r="L1" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="69" t="s">
+      <c r="M1" s="67" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="151.5" customHeight="1">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="42" t="s">
         <v>28</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="46" t="s">
+      <c r="F2" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="68" t="s">
+      <c r="G2" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="47" t="s">
+      <c r="H2" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="48" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="48" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="49">
+      <c r="I2" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="47">
         <v>46200</v>
       </c>
-      <c r="L2" s="66"/>
+      <c r="L2" s="64"/>
       <c r="M2" s="11" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="121.5">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="48" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="51" t="s">
+      <c r="B3" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="52" t="s">
+      <c r="C3" s="50" t="s">
         <v>35</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="53" t="s">
+      <c r="E3" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="54" t="s">
+      <c r="F3" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="G3" s="55" t="s">
+      <c r="G3" s="53" t="s">
         <v>18</v>
       </c>
       <c r="H3" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="56" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="57">
+      <c r="I3" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="54" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="55">
         <v>46201</v>
       </c>
-      <c r="L3" s="67"/>
+      <c r="L3" s="65"/>
       <c r="M3" s="11" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="120" customHeight="1">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="44" t="s">
+      <c r="B4" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="37" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="15" t="s">
@@ -2768,13 +3229,13 @@
       </c>
     </row>
     <row r="5" spans="1:14" ht="114.75" customHeight="1">
-      <c r="A5" s="58" t="s">
+      <c r="A5" s="56" t="s">
         <v>45</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="37" t="s">
         <v>41</v>
       </c>
       <c r="D5" s="15" t="s">
@@ -2792,10 +3253,10 @@
       <c r="H5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="23" t="s">
+      <c r="I5" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="22" t="s">
         <v>20</v>
       </c>
       <c r="K5" s="10">
@@ -2807,13 +3268,13 @@
       </c>
     </row>
     <row r="6" spans="1:14" ht="142.5" customHeight="1">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="41" t="s">
         <v>50</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="37" t="s">
         <v>41</v>
       </c>
       <c r="D6" s="18" t="s">
@@ -2831,29 +3292,29 @@
       <c r="H6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="23" t="s">
+      <c r="I6" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="22" t="s">
         <v>20</v>
       </c>
       <c r="K6" s="10">
         <v>46201</v>
       </c>
       <c r="L6" s="13"/>
-      <c r="M6" s="20" t="s">
+      <c r="M6" s="19" t="s">
         <v>55</v>
       </c>
       <c r="N6" s="3"/>
     </row>
     <row r="7" spans="1:14" ht="137.25">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="41" t="s">
         <v>56</v>
       </c>
       <c r="B7" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="37" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="18" t="s">
@@ -2871,10 +3332,10 @@
       <c r="H7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" s="23" t="s">
+      <c r="I7" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="22" t="s">
         <v>20</v>
       </c>
       <c r="K7" s="10">
@@ -2885,20 +3346,44 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
-      <c r="A8" s="19"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
+    <row r="8" spans="1:14" ht="96.75" customHeight="1">
+      <c r="A8" s="68" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I8" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K8" s="10">
+        <v>46203</v>
+      </c>
       <c r="L8" s="13"/>
-      <c r="M8" s="11"/>
+      <c r="M8" s="11" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="8"/>
@@ -2936,7 +3421,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2946,7 +3430,7 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="41.140625" customWidth="1"/>
     <col min="4" max="6" width="36.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
@@ -2958,61 +3442,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="17.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="37" t="s">
+      <c r="C1" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="37" t="s">
+      <c r="D1" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="38" t="s">
+      <c r="E1" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="38" t="s">
+      <c r="F1" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="37" t="s">
+      <c r="G1" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="37" t="s">
+      <c r="H1" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="37" t="s">
+      <c r="I1" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="37" t="s">
+      <c r="J1" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="37" t="s">
+      <c r="K1" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="37" t="s">
+      <c r="L1" s="35" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="101.25" customHeight="1">
       <c r="A2" s="11" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="C2" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="E2" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>66</v>
+        <v>68</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="19" t="s">
+        <v>72</v>
       </c>
       <c r="G2" s="11" t="s">
         <v>18</v>
@@ -3033,22 +3517,22 @@
     </row>
     <row r="3" spans="1:12" ht="105" customHeight="1">
       <c r="A3" s="11" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="D3" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="E3" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="F3" s="20" t="s">
-        <v>72</v>
+        <v>74</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>78</v>
       </c>
       <c r="G3" s="11" t="s">
         <v>18</v>
@@ -3067,32 +3551,76 @@
       </c>
       <c r="L3" s="11"/>
     </row>
-    <row r="4" spans="1:12">
-      <c r="A4" s="11"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
+    <row r="4" spans="1:12" ht="106.5">
+      <c r="A4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="12">
+        <v>46203</v>
+      </c>
       <c r="L4" s="11"/>
     </row>
-    <row r="5" spans="1:12">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
+    <row r="5" spans="1:12" ht="152.25">
+      <c r="A5" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="12">
+        <v>46203</v>
+      </c>
       <c r="L5" s="11"/>
     </row>
     <row r="6" spans="1:12">
@@ -3117,20 +3645,19 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03E9E5F8-86B1-40AA-A4FC-5C5ED968AE30}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="47" customWidth="1"/>
-    <col min="4" max="4" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="36.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="47.5703125" customWidth="1"/>
+    <col min="12" max="12" width="51.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="13.5" customHeight="1">
@@ -3146,10 +3673,10 @@
       <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="20" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="6" t="s">
@@ -3172,76 +3699,112 @@
       </c>
     </row>
     <row r="2" spans="1:12" ht="129" customHeight="1">
-      <c r="A2" s="30" t="s">
-        <v>73</v>
-      </c>
-      <c r="B2" s="31" t="s">
-        <v>74</v>
-      </c>
-      <c r="C2" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>76</v>
-      </c>
-      <c r="E2" s="31" t="s">
-        <v>77</v>
-      </c>
-      <c r="F2" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="G2" s="30" t="s">
+      <c r="A2" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="G2" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="30" t="s">
+      <c r="H2" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="34">
+      <c r="I2" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="33">
         <v>46200</v>
       </c>
-      <c r="L2" s="22"/>
+      <c r="L2" s="21"/>
     </row>
     <row r="3" spans="1:12" ht="103.5" customHeight="1">
-      <c r="A3" s="25" t="s">
-        <v>79</v>
-      </c>
-      <c r="B3" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3" s="27" t="s">
-        <v>75</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="E3" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="F3" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="G3" s="25" t="s">
+      <c r="A3" s="29" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="E3" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="F3" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="G3" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="35" t="s">
+      <c r="H3" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="36">
+      <c r="I3" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="70">
         <v>46200</v>
       </c>
-      <c r="L3" s="11"/>
+      <c r="L3" s="21"/>
+    </row>
+    <row r="4" spans="1:12" ht="148.5" customHeight="1">
+      <c r="A4" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="F4" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="G4" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="28">
+        <v>46203</v>
+      </c>
+      <c r="L4" s="62"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3251,7 +3814,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EF25B9E-3338-4408-8EB2-310117A2CBD5}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.140625" bestFit="1" customWidth="1"/>
@@ -3263,7 +3826,7 @@
     <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="52.7109375" customWidth="1"/>
+    <col min="12" max="12" width="71.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="20.25" customHeight="1">
@@ -3305,112 +3868,148 @@
       </c>
     </row>
     <row r="2" spans="1:12" ht="140.25" customHeight="1">
-      <c r="A2" s="25" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="26" t="s">
-        <v>85</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="D2" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="E2" s="26" t="s">
-        <v>88</v>
-      </c>
-      <c r="F2" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G2" s="25" t="s">
+      <c r="A2" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="G2" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="29">
+      <c r="I2" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="28">
         <v>46200</v>
       </c>
       <c r="L2" s="11"/>
     </row>
     <row r="3" spans="1:12" ht="143.25" customHeight="1">
-      <c r="A3" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>93</v>
-      </c>
-      <c r="E3" s="26" t="s">
-        <v>94</v>
-      </c>
-      <c r="F3" s="26" t="s">
-        <v>95</v>
-      </c>
-      <c r="G3" s="25" t="s">
+      <c r="A3" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="G3" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="29">
+      <c r="I3" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="28">
         <v>46200</v>
       </c>
       <c r="L3" s="11"/>
     </row>
     <row r="4" spans="1:12" ht="146.25" customHeight="1">
-      <c r="A4" s="25" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>97</v>
-      </c>
-      <c r="C4" s="27" t="s">
-        <v>98</v>
-      </c>
-      <c r="D4" s="26" t="s">
-        <v>99</v>
-      </c>
-      <c r="E4" s="26" t="s">
-        <v>100</v>
-      </c>
-      <c r="F4" s="26" t="s">
-        <v>101</v>
-      </c>
-      <c r="G4" s="25" t="s">
+      <c r="A4" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>123</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>124</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" s="29">
+      <c r="I4" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="33">
         <v>46200</v>
       </c>
-      <c r="L4" s="11"/>
+      <c r="L4" s="21"/>
+    </row>
+    <row r="5" spans="1:12" ht="135" customHeight="1">
+      <c r="A5" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="28">
+        <v>46203</v>
+      </c>
+      <c r="L5" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3420,13 +4019,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22552AF2-C7A2-43AD-9792-589143CF59CD}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.28515625" customWidth="1"/>
     <col min="3" max="3" width="26.140625" customWidth="1"/>
-    <col min="4" max="4" width="27" customWidth="1"/>
+    <col min="4" max="4" width="31" customWidth="1"/>
     <col min="5" max="5" width="36" customWidth="1"/>
     <col min="6" max="6" width="32.140625" customWidth="1"/>
     <col min="7" max="7" width="27.85546875" customWidth="1"/>
@@ -3450,10 +4049,10 @@
       <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="20" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="6" t="s">
@@ -3476,112 +4075,148 @@
       </c>
     </row>
     <row r="2" spans="1:12" ht="91.5">
-      <c r="A2" s="25" t="s">
-        <v>102</v>
-      </c>
-      <c r="B2" s="26" t="s">
-        <v>103</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>98</v>
-      </c>
-      <c r="D2" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="E2" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="F2" s="26" t="s">
-        <v>106</v>
-      </c>
-      <c r="G2" s="25" t="s">
+      <c r="A2" s="24" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="G2" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="63" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="63" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="29">
+      <c r="I2" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="28">
         <v>46200</v>
       </c>
-      <c r="L2" s="64"/>
+      <c r="L2" s="62"/>
     </row>
     <row r="3" spans="1:12" ht="152.25">
-      <c r="A3" s="25" t="s">
-        <v>107</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>109</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="E3" s="26" t="s">
-        <v>111</v>
-      </c>
-      <c r="F3" s="26" t="s">
-        <v>112</v>
-      </c>
-      <c r="G3" s="25" t="s">
+      <c r="A3" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>138</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="G3" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="63" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="63" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="29">
+      <c r="I3" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="28">
         <v>46200</v>
       </c>
-      <c r="L3" s="64"/>
+      <c r="L3" s="62"/>
     </row>
     <row r="4" spans="1:12" ht="134.25" customHeight="1">
-      <c r="A4" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>114</v>
-      </c>
-      <c r="C4" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="26" t="s">
-        <v>115</v>
-      </c>
-      <c r="E4" s="26" t="s">
-        <v>116</v>
-      </c>
-      <c r="F4" s="26" t="s">
-        <v>117</v>
-      </c>
-      <c r="G4" s="25" t="s">
+      <c r="A4" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>146</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="G4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="63" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="63" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" s="29">
+      <c r="I4" s="71" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="71" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="33">
         <v>46200</v>
       </c>
-      <c r="L4" s="64"/>
+      <c r="L4" s="72"/>
+    </row>
+    <row r="5" spans="1:12" ht="167.25">
+      <c r="A5" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>152</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="28">
+        <v>46203</v>
+      </c>
+      <c r="L5" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualizacion matriz casos de prueba
</commit_message>
<xml_diff>
--- a/documentacion/Matriz de casos de prueba.xlsx
+++ b/documentacion/Matriz de casos de prueba.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC40F387-DCCE-411D-B3AA-536B5CB1C21E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{269883D9-56C1-4B84-ADC1-050201D0B7AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14,6 +14,7 @@
     <sheet name="Movimientos" sheetId="4" r:id="rId4"/>
     <sheet name="Categorias" sheetId="5" r:id="rId5"/>
     <sheet name="Proveedores" sheetId="6" r:id="rId6"/>
+    <sheet name="Usuarios" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="J1K1">Dashboard!$J$1:$J$1</definedName>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="177">
   <si>
     <t>ID</t>
   </si>
@@ -172,6 +173,51 @@
   </si>
   <si>
     <t>El sistema permite el acceso y te dirige al Dashboard (home)</t>
+  </si>
+  <si>
+    <t>R-001</t>
+  </si>
+  <si>
+    <t>Registro Exitoso</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Ingresar a </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>https://challenge-tecnico-aranguri-apps.vercel.app/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve"> y presionar registrarse</t>
+    </r>
+  </si>
+  <si>
+    <t>1- Completar Nombre completo con "Juan Pérez"  2- Completar Email con uno no registrado
+3- Completar Contraseña con "Test1234"
+4- Completar Confirmar contraseña con "Test1234"
+5- Click en "Crear cuenta"</t>
+  </si>
+  <si>
+    <t>El sistema crea la cuenta correctamente</t>
+  </si>
+  <si>
+    <t>El sistema permite el acceso y te dirige al Dashboard (home), o muestra mensaje de confirmación</t>
   </si>
   <si>
     <t>Derivados</t>
@@ -362,6 +408,30 @@
     <t>El sistema muestra correctamente el mensaje Buenas tardes, Admin y el subtitulo Resumen general del inventario.</t>
   </si>
   <si>
+    <t>DB-008</t>
+  </si>
+  <si>
+    <t>Reescalado automático del eje Y en gráfico de Movimientos</t>
+  </si>
+  <si>
+    <t>Ingresar a https://challenge-tecnico-aranguri-apps.vercel.app/ con credenciales: Mail: Admin@email.com Password: Admin123. Ubicarse en el Dashboard, gráfico de Movimientos con rango 7d, eje Y con tope actual en 8.</t>
+  </si>
+  <si>
+    <t>1- Ir al modulo de Movimientos.
+2- Registrar entradas, salidas o ajustes hasta superar el valor de 4 en un mismo dia (del mismo tipo).
+3- Volver al Dashboard.
+4- Observar el grafico de Movimientos en el rango 7d.</t>
+  </si>
+  <si>
+    <t>El eje Y del grafico se reescala automaticamente para acomodar el nuevo valor maximo, mostrando la curva completa sin recortes.</t>
+  </si>
+  <si>
+    <t>El eje Y pasa de un tope de 4 a un tope superior de 8 reflejando el nuevo maximo de movimientos registrados.</t>
+  </si>
+  <si>
+    <t>UI</t>
+  </si>
+  <si>
     <t>PR-001</t>
   </si>
   <si>
@@ -491,9 +561,6 @@
     <t>El panel se despliega correctamente, todos los campos son visibles, los obligatorios tienen asterisco y el boton es amarillo.</t>
   </si>
   <si>
-    <t>UI</t>
-  </si>
-  <si>
     <t>MOV-001</t>
   </si>
   <si>
@@ -788,12 +855,49 @@
   <si>
     <t>El proveedor Distribuidora Sur SA se guarda y aparece en la grilla con el contacto, email y telefono correctos.</t>
   </si>
+  <si>
+    <t>USR-001</t>
+  </si>
+  <si>
+    <t>Editar rol de usuario exitosamente</t>
+  </si>
+  <si>
+    <t>Ingresar a https://challenge-tecnico-aranguri-apps.vercel.app/ con credenciales: Mail: Admin@email.com Password: Admin123. Navegar al módulo de Usuarios.</t>
+  </si>
+  <si>
+    <t>1- Ubicar el usuario prueba@email.com.
+2- Hacer click en el desplegable de Rol (actualmente Lectura).
+3- Seleccionar el rol Encargado.</t>
+  </si>
+  <si>
+    <t>El rol del usuario se actualiza correctamente y se refleja en la grilla sin necesidad de recargar la página.</t>
+  </si>
+  <si>
+    <t>El usuario prueba@email.com pasa a tener el rol Encargado.</t>
+  </si>
+  <si>
+    <t>USR-002</t>
+  </si>
+  <si>
+    <t>Eliminar usuario exitosamente</t>
+  </si>
+  <si>
+    <t>1- Ubicar el usuario prueba@email.com.
+2- Hacer click en el ícono de papelera (eliminar).
+3- Confirmar la eliminación si el sistema solicita confirmación.</t>
+  </si>
+  <si>
+    <t>El usuario se elimina correctamente y desaparece de la grilla.</t>
+  </si>
+  <si>
+    <t>El usuario prueba@email.com ya no aparece en la lista de Usuarios.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -883,6 +987,10 @@
       <color theme="0"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1057,7 +1165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1068,64 +1176,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1159,72 +1221,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1241,23 +1246,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1269,6 +1265,105 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1387,6 +1482,53 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2209800</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1895475</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A927412-06DC-1DC1-664E-935169A4B0C1}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{90273EA4-FF72-41AD-E852-7F672C06DE97}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15925800" y="3848100"/>
+          <a:ext cx="1562100" cy="1838325"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1757,6 +1899,53 @@
         <a:xfrm>
           <a:off x="17849850" y="10220325"/>
           <a:ext cx="2752725" cy="1209675"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1219200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>3276600</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>1228725</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Imagen 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E3152D4D-09C4-64E8-A6EF-E15B847053AA}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{7D6E3768-50E7-D321-DC1E-747AEDCE56CD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18154650" y="11439525"/>
+          <a:ext cx="2590800" cy="1238250"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2611,6 +2800,102 @@
         <a:xfrm flipV="1">
           <a:off x="16154400" y="5886450"/>
           <a:ext cx="1914525" cy="504825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>390525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>1219200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED7E5D9E-37C9-4B29-51D9-B06B326ED49C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13963650" y="819150"/>
+          <a:ext cx="2762250" cy="828675"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>323850</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2771775</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>1162050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FABAE959-F3C7-14F7-EB13-EB9C8A5CEDA7}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{ED7E5D9E-37C9-4B29-51D9-B06B326ED49C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14049375" y="2295525"/>
+          <a:ext cx="2581275" cy="838200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2919,131 +3204,183 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1071EF2-3E39-441E-A0A9-CEDA178FF542}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.42578125" customWidth="1"/>
-    <col min="5" max="6" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="43.42578125" customWidth="1"/>
+    <col min="1" max="1" width="6" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.42578125" style="29" customWidth="1"/>
+    <col min="5" max="6" width="36.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="43.42578125" style="29" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="20" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="147" customHeight="1">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="57" t="s">
+      <c r="C2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="30" t="s">
+      <c r="D2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="30" t="s">
+      <c r="E2" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="73" t="s">
+      <c r="F2" s="68" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="29" t="s">
+      <c r="G2" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="29" t="s">
+      <c r="H2" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="33">
+      <c r="I2" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="17">
         <v>46201</v>
       </c>
-      <c r="L2" s="21"/>
+      <c r="L2" s="13"/>
     </row>
     <row r="3" spans="1:12" ht="117.75" customHeight="1">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="58" t="s">
+      <c r="C3" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="D3" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="60" t="s">
+      <c r="F3" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="G3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="28">
+      <c r="I3" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="12">
         <v>46202</v>
       </c>
-      <c r="L3" s="4"/>
+      <c r="L3" s="66"/>
+    </row>
+    <row r="5" spans="1:12" ht="151.5" customHeight="1">
+      <c r="A5" s="42" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="12">
+        <v>46203</v>
+      </c>
+      <c r="L5" s="8"/>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="C11" s="30"/>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="C12" s="30"/>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="C13" s="30"/>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="C14" s="30"/>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="C15" s="30"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3071,181 +3408,181 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="17.25">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="38" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="39" t="s">
+      <c r="D1" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="F1" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="39" t="s">
+      <c r="G1" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="38" t="s">
+      <c r="H1" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="38" t="s">
+      <c r="I1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="38" t="s">
+      <c r="J1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="39" t="s">
+      <c r="K1" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="63" t="s">
+      <c r="L1" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="67" t="s">
-        <v>26</v>
+      <c r="M1" s="28" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="151.5" customHeight="1">
-      <c r="A2" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" s="42" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="43" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="44" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" s="44" t="s">
-        <v>32</v>
-      </c>
-      <c r="G2" s="66" t="s">
+      <c r="A2" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="45" t="s">
+      <c r="H2" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="47">
+      <c r="I2" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="52">
         <v>46200</v>
       </c>
-      <c r="L2" s="64"/>
-      <c r="M2" s="11" t="s">
+      <c r="L2" s="53"/>
+      <c r="M2" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="121.5">
-      <c r="A3" s="48" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" s="49" t="s">
-        <v>34</v>
-      </c>
-      <c r="C3" s="50" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" s="51" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" s="52" t="s">
-        <v>38</v>
-      </c>
-      <c r="G3" s="53" t="s">
+      <c r="A3" s="54" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" s="57" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="58" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="H3" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="54" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="55">
+      <c r="I3" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="59" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="19">
         <v>46201</v>
       </c>
-      <c r="L3" s="65"/>
-      <c r="M3" s="11" t="s">
+      <c r="L3" s="18"/>
+      <c r="M3" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="120" customHeight="1">
-      <c r="A4" s="41" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="37" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>44</v>
+      <c r="A4" s="45" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="61" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="61" t="s">
+        <v>50</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" s="10">
+      <c r="I4" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="12">
         <v>46201</v>
       </c>
-      <c r="L4" s="13"/>
-      <c r="M4" s="11" t="s">
+      <c r="L4" s="18"/>
+      <c r="M4" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="114.75" customHeight="1">
-      <c r="A5" s="56" t="s">
-        <v>45</v>
+      <c r="A5" s="63" t="s">
+        <v>51</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="37" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>49</v>
+      <c r="D5" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>18</v>
@@ -3253,38 +3590,38 @@
       <c r="H5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5" s="10">
+      <c r="I5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="12">
         <v>46201</v>
       </c>
-      <c r="L5" s="13"/>
-      <c r="M5" s="11" t="s">
+      <c r="L5" s="18"/>
+      <c r="M5" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="142.5" customHeight="1">
-      <c r="A6" s="41" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="37" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>54</v>
+      <c r="A6" s="45" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>60</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>18</v>
@@ -3292,39 +3629,39 @@
       <c r="H6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="K6" s="10">
+      <c r="I6" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" s="12">
         <v>46201</v>
       </c>
-      <c r="L6" s="13"/>
-      <c r="M6" s="19" t="s">
-        <v>55</v>
+      <c r="L6" s="18"/>
+      <c r="M6" s="9" t="s">
+        <v>61</v>
       </c>
       <c r="N6" s="3"/>
     </row>
     <row r="7" spans="1:14" ht="137.25">
-      <c r="A7" s="41" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="37" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>60</v>
+      <c r="A7" s="45" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>66</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>18</v>
@@ -3332,73 +3669,97 @@
       <c r="H7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="K7" s="10">
+      <c r="I7" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K7" s="12">
         <v>46201</v>
       </c>
-      <c r="L7" s="13"/>
-      <c r="M7" s="11" t="s">
+      <c r="L7" s="18"/>
+      <c r="M7" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="96.75" customHeight="1">
-      <c r="A8" s="68" t="s">
-        <v>61</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="G8" s="8" t="s">
+      <c r="A8" s="64" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="K8" s="10">
+      <c r="I8" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="K8" s="17">
         <v>46203</v>
       </c>
-      <c r="L8" s="13"/>
-      <c r="M8" s="11" t="s">
+      <c r="L8" s="31"/>
+      <c r="M8" s="13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="11"/>
+    <row r="9" spans="1:14" ht="101.25" customHeight="1">
+      <c r="A9" s="41" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="41" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="41" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="41" t="s">
+        <v>78</v>
+      </c>
+      <c r="G9" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="H9" s="43" t="s">
+        <v>79</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9" s="44">
+        <v>46203</v>
+      </c>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="3"/>
@@ -3429,151 +3790,152 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.140625" customWidth="1"/>
-    <col min="4" max="6" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="40.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.140625" style="29" customWidth="1"/>
+    <col min="4" max="6" width="36.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="40.42578125" style="29" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="17.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="36" t="s">
+      <c r="E1" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="F1" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="35" t="s">
+      <c r="G1" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="35" t="s">
+      <c r="H1" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="35" t="s">
+      <c r="I1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="35" t="s">
+      <c r="J1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="35" t="s">
+      <c r="K1" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="35" t="s">
+      <c r="L1" s="20" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="101.25" customHeight="1">
-      <c r="A2" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="D2" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="F2" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="G2" s="11" t="s">
+      <c r="A2" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="14" t="s">
+      <c r="I2" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="11" t="s">
         <v>20</v>
       </c>
       <c r="K2" s="12">
         <v>46201</v>
       </c>
-      <c r="L2" s="11"/>
+      <c r="L2" s="8"/>
     </row>
     <row r="3" spans="1:12" ht="105" customHeight="1">
-      <c r="A3" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="D3" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="F3" s="19" t="s">
-        <v>78</v>
-      </c>
-      <c r="G3" s="11" t="s">
+      <c r="A3" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="14" t="s">
+      <c r="I3" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="11" t="s">
         <v>20</v>
       </c>
       <c r="K3" s="12">
         <v>46202</v>
       </c>
-      <c r="L3" s="11"/>
+      <c r="L3" s="8"/>
     </row>
     <row r="4" spans="1:12" ht="106.5">
-      <c r="A4" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="F4" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="G4" s="11" t="s">
+      <c r="A4" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="G4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="8" t="s">
         <v>19</v>
       </c>
       <c r="I4" s="11" t="s">
@@ -3585,32 +3947,32 @@
       <c r="K4" s="12">
         <v>46203</v>
       </c>
-      <c r="L4" s="11"/>
+      <c r="L4" s="8"/>
     </row>
     <row r="5" spans="1:12" ht="152.25">
-      <c r="A5" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="F5" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="G5" s="11" t="s">
+      <c r="A5" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="G5" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="11" t="s">
-        <v>90</v>
+      <c r="H5" s="13" t="s">
+        <v>79</v>
       </c>
       <c r="I5" s="11" t="s">
         <v>20</v>
@@ -3618,24 +3980,24 @@
       <c r="J5" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="17">
         <v>46203</v>
       </c>
-      <c r="L5" s="11"/>
+      <c r="L5" s="13"/>
     </row>
     <row r="6" spans="1:12">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
+      <c r="A6" s="67"/>
+      <c r="B6" s="67"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="67"/>
+      <c r="G6" s="67"/>
+      <c r="H6" s="67"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="67"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="67"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3661,150 +4023,150 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="13.5" customHeight="1">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="129" customHeight="1">
-      <c r="A2" s="29" t="s">
-        <v>91</v>
-      </c>
-      <c r="B2" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="D2" s="30" t="s">
-        <v>94</v>
-      </c>
-      <c r="E2" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="F2" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="G2" s="29" t="s">
+      <c r="A2" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="G2" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="29" t="s">
+      <c r="H2" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="33">
+      <c r="I2" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="17">
         <v>46200</v>
       </c>
-      <c r="L2" s="21"/>
+      <c r="L2" s="7"/>
     </row>
     <row r="3" spans="1:12" ht="103.5" customHeight="1">
-      <c r="A3" s="29" t="s">
-        <v>97</v>
-      </c>
-      <c r="B3" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="C3" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="D3" s="30" t="s">
-        <v>99</v>
-      </c>
-      <c r="E3" s="30" t="s">
-        <v>100</v>
-      </c>
-      <c r="F3" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="G3" s="29" t="s">
+      <c r="A3" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="G3" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="69" t="s">
+      <c r="H3" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="70">
+      <c r="I3" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="32">
         <v>46200</v>
       </c>
-      <c r="L3" s="21"/>
+      <c r="L3" s="7"/>
     </row>
     <row r="4" spans="1:12" ht="148.5" customHeight="1">
-      <c r="A4" s="24" t="s">
-        <v>102</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>105</v>
-      </c>
-      <c r="E4" s="25" t="s">
-        <v>106</v>
-      </c>
-      <c r="F4" s="25" t="s">
-        <v>107</v>
-      </c>
-      <c r="G4" s="24" t="s">
+      <c r="A4" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="G4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="H4" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" s="28">
+      <c r="I4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="12">
         <v>46203</v>
       </c>
-      <c r="L4" s="62"/>
+      <c r="L4" s="27"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3868,148 +4230,148 @@
       </c>
     </row>
     <row r="2" spans="1:12" ht="140.25" customHeight="1">
-      <c r="A2" s="24" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>109</v>
-      </c>
-      <c r="C2" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" s="25" t="s">
-        <v>111</v>
-      </c>
-      <c r="E2" s="25" t="s">
-        <v>112</v>
-      </c>
-      <c r="F2" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="G2" s="24" t="s">
+      <c r="A2" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="G2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="24" t="s">
+      <c r="H2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="28">
+      <c r="I2" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="12">
         <v>46200</v>
       </c>
-      <c r="L2" s="11"/>
+      <c r="L2" s="5"/>
     </row>
     <row r="3" spans="1:12" ht="143.25" customHeight="1">
-      <c r="A3" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="B3" s="25" t="s">
-        <v>115</v>
-      </c>
-      <c r="C3" s="25" t="s">
-        <v>116</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>118</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>119</v>
-      </c>
-      <c r="G3" s="24" t="s">
+      <c r="A3" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="G3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="28">
+      <c r="I3" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="12">
         <v>46200</v>
       </c>
-      <c r="L3" s="11"/>
+      <c r="L3" s="5"/>
     </row>
     <row r="4" spans="1:12" ht="146.25" customHeight="1">
-      <c r="A4" s="29" t="s">
-        <v>120</v>
-      </c>
-      <c r="B4" s="30" t="s">
-        <v>121</v>
-      </c>
-      <c r="C4" s="31" t="s">
-        <v>122</v>
-      </c>
-      <c r="D4" s="30" t="s">
-        <v>123</v>
-      </c>
-      <c r="E4" s="30" t="s">
-        <v>124</v>
-      </c>
-      <c r="F4" s="30" t="s">
-        <v>125</v>
-      </c>
-      <c r="G4" s="29" t="s">
+      <c r="A4" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="G4" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="29" t="s">
+      <c r="H4" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" s="33">
+      <c r="I4" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="17">
         <v>46200</v>
       </c>
-      <c r="L4" s="21"/>
+      <c r="L4" s="7"/>
     </row>
     <row r="5" spans="1:12" ht="135" customHeight="1">
-      <c r="A5" s="24" t="s">
-        <v>126</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>127</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>128</v>
-      </c>
-      <c r="D5" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="F5" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="G5" s="24" t="s">
+      <c r="A5" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="G5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="24" t="s">
+      <c r="H5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5" s="28">
+      <c r="I5" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="12">
         <v>46203</v>
       </c>
-      <c r="L5" s="24"/>
+      <c r="L5" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4037,186 +4399,321 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21" customHeight="1">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="91.5">
-      <c r="A2" s="24" t="s">
-        <v>132</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>133</v>
-      </c>
-      <c r="C2" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="D2" s="25" t="s">
+      <c r="A2" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="E2" s="25" t="s">
-        <v>135</v>
-      </c>
-      <c r="F2" s="25" t="s">
-        <v>136</v>
-      </c>
-      <c r="G2" s="24" t="s">
+      <c r="D2" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="G2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="24" t="s">
+      <c r="H2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="61" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="61" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="28">
+      <c r="I2" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="12">
         <v>46200</v>
       </c>
-      <c r="L2" s="62"/>
+      <c r="L2" s="27"/>
     </row>
     <row r="3" spans="1:12" ht="152.25">
-      <c r="A3" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="B3" s="25" t="s">
-        <v>138</v>
-      </c>
-      <c r="C3" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>140</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>141</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>142</v>
-      </c>
-      <c r="G3" s="24" t="s">
+      <c r="A3" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="G3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="61" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="61" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="28">
+      <c r="I3" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="12">
         <v>46200</v>
       </c>
-      <c r="L3" s="62"/>
+      <c r="L3" s="27"/>
     </row>
     <row r="4" spans="1:12" ht="134.25" customHeight="1">
-      <c r="A4" s="29" t="s">
-        <v>143</v>
-      </c>
-      <c r="B4" s="30" t="s">
-        <v>144</v>
-      </c>
-      <c r="C4" s="31" t="s">
-        <v>110</v>
-      </c>
-      <c r="D4" s="30" t="s">
-        <v>145</v>
-      </c>
-      <c r="E4" s="30" t="s">
-        <v>146</v>
-      </c>
-      <c r="F4" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="G4" s="29" t="s">
+      <c r="A4" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="G4" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="29" t="s">
+      <c r="H4" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="71" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="71" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" s="33">
+      <c r="I4" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="17">
         <v>46200</v>
       </c>
-      <c r="L4" s="72"/>
+      <c r="L4" s="34"/>
     </row>
     <row r="5" spans="1:12" ht="167.25">
-      <c r="A5" s="24" t="s">
-        <v>148</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>149</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>150</v>
-      </c>
-      <c r="D5" s="25" t="s">
-        <v>151</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>152</v>
-      </c>
-      <c r="F5" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="G5" s="24" t="s">
+      <c r="A5" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="G5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="24" t="s">
+      <c r="H5" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5" s="28">
+      <c r="I5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="19">
         <v>46203</v>
       </c>
-      <c r="L5" s="24"/>
+      <c r="L5" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80983849-66D8-432F-AA92-8EB2E00764F9}">
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="42" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="33.75">
+      <c r="A1" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="37" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="38" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="38" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="37" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="37" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="37" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="37" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="37" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="121.5">
+      <c r="A2" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" s="39" t="s">
+        <v>167</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="17">
+        <v>46203</v>
+      </c>
+      <c r="L2" s="13"/>
+    </row>
+    <row r="3" spans="1:12" ht="102" customHeight="1">
+      <c r="A3" s="40" t="s">
+        <v>172</v>
+      </c>
+      <c r="B3" s="41" t="s">
+        <v>173</v>
+      </c>
+      <c r="C3" s="41" t="s">
+        <v>168</v>
+      </c>
+      <c r="D3" s="41" t="s">
+        <v>174</v>
+      </c>
+      <c r="E3" s="41" t="s">
+        <v>175</v>
+      </c>
+      <c r="F3" s="41" t="s">
+        <v>176</v>
+      </c>
+      <c r="G3" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="44">
+        <v>46203</v>
+      </c>
+      <c r="L3" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>